<commit_message>
tests and improvenments of client
</commit_message>
<xml_diff>
--- a/docs/container-support.xlsx
+++ b/docs/container-support.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$L$48</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$L$49</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="153">
   <si>
     <t xml:space="preserve">FastCacheAsyncSimpleClient</t>
   </si>
@@ -476,6 +476,12 @@
   </si>
   <si>
     <t xml:space="preserve">Добавление элементов в карты</t>
+  </si>
+  <si>
+    <t xml:space="preserve">streamElementInRangeOrderedMap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Потоковый экспорт элементов в диапазоне</t>
   </si>
 </sst>
 </file>
@@ -485,7 +491,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -506,6 +512,18 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF080808"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -550,7 +568,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -563,6 +581,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -572,7 +598,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -580,7 +606,75 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF080808"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF080808"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -696,19 +790,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="true">
+  <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="48.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="55.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="40.67"/>
   </cols>
   <sheetData>
@@ -826,7 +922,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -840,7 +936,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
@@ -854,7 +950,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
@@ -868,7 +964,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
@@ -1020,7 +1116,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>43</v>
       </c>
@@ -1033,11 +1129,14 @@
       <c r="E12" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="F12" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="L12" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
         <v>46</v>
       </c>
@@ -1050,11 +1149,14 @@
       <c r="E13" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="F13" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="L13" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>49</v>
       </c>
@@ -1074,7 +1176,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
         <v>52</v>
       </c>
@@ -1088,6 +1190,9 @@
         <v>14</v>
       </c>
       <c r="H15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J15" s="1" t="s">
         <v>14</v>
       </c>
       <c r="L15" s="1" t="s">
@@ -1124,7 +1229,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
         <v>58</v>
       </c>
@@ -1147,16 +1252,14 @@
         <v>60</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1" t="s">
         <v>14</v>
@@ -1170,13 +1273,11 @@
       <c r="H18" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
       <c r="L18" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
         <v>64</v>
       </c>
@@ -1193,7 +1294,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
         <v>67</v>
       </c>
@@ -1213,7 +1314,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
         <v>70</v>
       </c>
@@ -1230,7 +1331,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
         <v>72</v>
       </c>
@@ -1247,7 +1348,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
         <v>75</v>
       </c>
@@ -1264,7 +1365,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
         <v>78</v>
       </c>
@@ -1280,11 +1381,14 @@
       <c r="H24" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="J24" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="L24" s="1" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
         <v>81</v>
       </c>
@@ -1304,7 +1408,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
         <v>84</v>
       </c>
@@ -1317,11 +1421,14 @@
       <c r="E26" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="F26" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="L26" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>87</v>
       </c>
@@ -1380,9 +1487,6 @@
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
       <c r="I29" s="1" t="s">
         <v>14</v>
       </c>
@@ -1469,7 +1573,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
         <v>101</v>
       </c>
@@ -1483,7 +1587,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
         <v>104</v>
       </c>
@@ -1497,7 +1601,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
         <v>107</v>
       </c>
@@ -1511,7 +1615,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
         <v>110</v>
       </c>
@@ -1525,7 +1629,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
         <v>113</v>
       </c>
@@ -1539,7 +1643,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
         <v>116</v>
       </c>
@@ -1553,7 +1657,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
         <v>119</v>
       </c>
@@ -1567,7 +1671,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
         <v>122</v>
       </c>
@@ -1581,7 +1685,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
         <v>125</v>
       </c>
@@ -1595,7 +1699,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
         <v>128</v>
       </c>
@@ -1609,7 +1713,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
         <v>131</v>
       </c>
@@ -1737,14 +1841,22 @@
         <v>150</v>
       </c>
     </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="J49" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L49" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L48">
-    <filterColumn colId="8">
-      <filters>
-        <filter val="✔"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:L49"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
massive update tests and interfaces cleanup
</commit_message>
<xml_diff>
--- a/docs/container-support.xlsx
+++ b/docs/container-support.xlsx
@@ -5,13 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="api capcbilities" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="tests" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$L$49</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'api capcbilities'!$A$1:$L$49</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="165">
   <si>
     <t xml:space="preserve">FastCacheAsyncSimpleClient</t>
   </si>
@@ -482,6 +483,42 @@
   </si>
   <si>
     <t xml:space="preserve">Потоковый экспорт элементов в диапазоне</t>
+  </si>
+  <si>
+    <t xml:space="preserve">simple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cluster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AtomicOperationsTest.java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HashMapOperationsTest.java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ListOperationsTest.java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OrderedMapOperationsTest.java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OrderedSetOperationsTest.java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QueueOperationsTest.java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SetOperationsTest.java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VectorOperationsTest.java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RawValuesTest.java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RawValuesClusterTest.java</t>
   </si>
 </sst>
 </file>
@@ -526,12 +563,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF81D41A"/>
+        <bgColor rgb="FF969696"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -568,7 +611,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -586,6 +629,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -659,7 +706,7 @@
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FF81D41A"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
@@ -790,7 +837,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
+  <sheetPr filterMode="true">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L49"/>
@@ -922,7 +969,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -936,7 +983,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
@@ -950,7 +997,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
@@ -964,7 +1011,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
@@ -1116,7 +1163,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>43</v>
       </c>
@@ -1136,7 +1183,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
         <v>46</v>
       </c>
@@ -1156,7 +1203,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>49</v>
       </c>
@@ -1252,7 +1299,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
         <v>61</v>
       </c>
@@ -1277,7 +1324,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
         <v>64</v>
       </c>
@@ -1294,7 +1341,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
         <v>67</v>
       </c>
@@ -1314,7 +1361,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
         <v>70</v>
       </c>
@@ -1331,7 +1378,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
         <v>72</v>
       </c>
@@ -1348,7 +1395,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
         <v>75</v>
       </c>
@@ -1388,7 +1435,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
         <v>81</v>
       </c>
@@ -1408,7 +1455,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
         <v>84</v>
       </c>
@@ -1428,7 +1475,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>87</v>
       </c>
@@ -1573,7 +1620,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
         <v>101</v>
       </c>
@@ -1587,7 +1634,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
         <v>104</v>
       </c>
@@ -1601,7 +1648,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
         <v>107</v>
       </c>
@@ -1615,7 +1662,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
         <v>110</v>
       </c>
@@ -1629,7 +1676,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
         <v>113</v>
       </c>
@@ -1643,7 +1690,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
         <v>116</v>
       </c>
@@ -1657,7 +1704,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
         <v>119</v>
       </c>
@@ -1671,7 +1718,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
         <v>122</v>
       </c>
@@ -1685,7 +1732,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
         <v>125</v>
       </c>
@@ -1699,7 +1746,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
         <v>128</v>
       </c>
@@ -1713,7 +1760,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
         <v>131</v>
       </c>
@@ -1856,7 +1903,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L49"/>
+  <autoFilter ref="A1:L49">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="✔"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1866,4 +1919,107 @@
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="27.88"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>164</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>